<commit_message>
feat: complete real enterprise data integration
</commit_message>
<xml_diff>
--- a/data/bom.xlsx
+++ b/data/bom.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="Rab0a2ff2bc004f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R9bbd7fed11944bd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BomData" displayName="BomData" ref="A1:C4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BomData" displayName="BomData" ref="A1:C6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="parent_material"/>
     <x:tableColumn id="2" name="child_material"/>
@@ -406,7 +406,7 @@
         <x:v>ABC-1000</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
-        <x:v>主板</x:v>
+        <x:v>控制模块</x:v>
       </x:c>
       <x:c r="C2" s="21" t="n">
         <x:v>1</x:v>
@@ -424,20 +424,42 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="8" t="str">
+      <x:c r="A4" s="6" t="str">
         <x:v>ABC-1000</x:v>
       </x:c>
-      <x:c r="B4" s="22" t="str">
+      <x:c r="B4" s="20" t="str">
         <x:v>螺丝</x:v>
       </x:c>
-      <x:c r="C4" s="23" t="n">
+      <x:c r="C4" s="21" t="n">
         <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>控制模块</x:v>
+      </x:c>
+      <x:c r="B5" s="20" t="str">
+        <x:v>主板</x:v>
+      </x:c>
+      <x:c r="C5" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>控制模块</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>芯片</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra84f35c958334a52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b0395ffff924d33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>